<commit_message>
Auto update Pengadaan 2026-10-09 08:09:33
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-09).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-09).xlsx
@@ -1020,35 +1020,27 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>1796500000</v>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1389,22 +1381,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>677290237</v>
+        <v>674360508</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>137583844</v>
+        <v>134654115</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>116218702</v>
+        <v>1345382085</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1426,13 +1418,13 @@
         <v>39</v>
       </c>
       <c r="D26" s="9" t="n">
-        <v>544252460</v>
+        <v>544171011</v>
       </c>
       <c r="E26" s="7" t="n">
         <v>17</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>350423349</v>
+        <v>350341900</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>17</v>
@@ -1528,13 +1520,13 @@
         <v>172</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2271451073</v>
+        <v>2261946920</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1136240668</v>
+        <v>1126736515</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1559,22 +1551,22 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>367878502</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>79101092</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>75945607</v>
+        <v>225945607</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>49</v>
@@ -1701,22 +1693,22 @@
         <v>2184236820</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F34" s="9" t="n">
-        <v>372735637</v>
+        <v>378335637</v>
       </c>
       <c r="G34" s="7" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>367296417</v>
+        <v>372846417</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J34" s="9" t="n">
-        <v>1811501183</v>
+        <v>1805901183</v>
       </c>
     </row>
     <row r="35" ht="45" customHeight="1">
@@ -1800,13 +1792,13 @@
         <v>95</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>858385693</v>
+        <v>817027093</v>
       </c>
       <c r="E37" s="4" t="n">
         <v>16</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>461686502</v>
+        <v>420327902</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>16</v>
@@ -1868,13 +1860,13 @@
         <v>112</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1305525621</v>
+        <v>1279995621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>18</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>378058156</v>
+        <v>352528156</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>18</v>
@@ -1905,22 +1897,22 @@
         <v>890594163</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F40" s="9" t="n">
-        <v>619933379</v>
+        <v>633345189</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>525416551</v>
+        <v>535599741</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="J40" s="9" t="n">
-        <v>270660784</v>
+        <v>257248974</v>
       </c>
     </row>
     <row r="41" ht="45" customHeight="1">
@@ -2035,22 +2027,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>141795000</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>64745634</v>
+        <v>75645612</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>17</v>
@@ -2355,30 +2347,24 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>111669795</v>
       </c>
-      <c r="E52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E52" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>68020787</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>14</v>
@@ -3334,25 +3320,25 @@
         <v>156</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>1487886270</v>
+        <v>1481524170</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>198895843</v>
+        <v>218178226</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>171985038</v>
+        <v>194745366</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J76" s="9" t="n">
-        <v>1288990427</v>
+        <v>1263345944</v>
       </c>
     </row>
     <row r="77" ht="45" customHeight="1">
@@ -3363,28 +3349,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3914</v>
+        <v>3945</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32592278796</v>
+        <v>32506512765</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>420</v>
+        <v>458</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6737094380</v>
+        <v>6695984642</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>420</v>
+        <v>458</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>6201325511.6</v>
+        <v>9494403177.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3494</v>
+        <v>3487</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>25855184416</v>
+        <v>25810528123</v>
       </c>
     </row>
   </sheetData>
@@ -3805,13 +3791,13 @@
         <v>5</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>428765330</v>
+        <v>413165330</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>276710330</v>
+        <v>261110330</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>3</v>
@@ -4606,28 +4592,28 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>1566751699</v>
+        <v>1346095756</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>1225542538</v>
+        <v>1004886595</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>896262562</v>
+        <v>852531955</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>896262562</v>
+        <v>852531955</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>4</v>
@@ -4848,28 +4834,28 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>538286000</v>
+        <v>388286000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>288750000</v>
+        <v>138750000</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
@@ -5584,28 +5570,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>595373450</v>
+        <v>523391100</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>417917650</v>
+        <v>345935300</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -6048,28 +6034,40 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>660566066</v>
-      </c>
-      <c r="E52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F52" s="9" t="n">
-        <v>340582172</v>
-      </c>
-      <c r="G52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" s="9" t="n">
-        <v>68020787</v>
-      </c>
-      <c r="I52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="J52" s="9" t="n">
-        <v>68020787</v>
+        <v>319983894</v>
+      </c>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K52" s="10" t="inlineStr">
         <is>
@@ -7536,28 +7534,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>827</v>
+        <v>820</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>97964756558</v>
+        <v>97165936093</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>65396508145</v>
+        <v>64597687680</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>63678192262.41</v>
+        <v>63405540890.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>37551167518.02</v>
+        <v>37278516146.02</v>
       </c>
       <c r="K77" s="12" t="n">
         <v>12</v>
@@ -8371,28 +8369,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>26395646241</v>
+        <v>24599146241</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>26395646241</v>
+        <v>24599146241</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8590,13 +8588,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8815,34 +8813,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>48003814160</v>
+        <v>5652342335</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>47632716881</v>
+        <v>5281245056</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>2945468782</v>
+        <v>1854621974</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -12013,34 +12011,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>240</v>
+        <v>216</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>180959034603</v>
+        <v>136523671866</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>159</v>
+        <v>135</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>143584386443</v>
+        <v>99149023706</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>159</v>
+        <v>135</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>70262150313.01001</v>
+        <v>67280217537.01</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>141</v>
+        <v>117</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>65813716513</v>
+        <v>62831783737</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>4005987066</v>
+        <v>2915140258</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>81</v>

</xml_diff>

<commit_message>
Auto update Pengadaan 2026-10-09 12:09:02
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-09).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-09).xlsx
@@ -1020,27 +1020,35 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
-        <v>1</v>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
-        <v>1</v>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>1796500000</v>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1381,22 +1389,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>128</v>
+        <v>103</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>674360508</v>
+        <v>677290237</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>134654115</v>
+        <v>137583844</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>1345382085</v>
+        <v>116218702</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1418,13 +1426,13 @@
         <v>39</v>
       </c>
       <c r="D26" s="9" t="n">
-        <v>544171011</v>
+        <v>544252460</v>
       </c>
       <c r="E26" s="7" t="n">
         <v>17</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>350341900</v>
+        <v>350423349</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>17</v>
@@ -1520,13 +1528,13 @@
         <v>172</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2261946920</v>
+        <v>2271451073</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1126736515</v>
+        <v>1136240668</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1551,22 +1559,22 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>367878502</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>79101092</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>225945607</v>
+        <v>75945607</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>49</v>
@@ -1792,13 +1800,13 @@
         <v>95</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>817027093</v>
+        <v>858385693</v>
       </c>
       <c r="E37" s="4" t="n">
         <v>16</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>420327902</v>
+        <v>461686502</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>16</v>
@@ -1860,13 +1868,13 @@
         <v>112</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1279995621</v>
+        <v>1305525621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>18</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>352528156</v>
+        <v>378058156</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>18</v>
@@ -2027,22 +2035,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>141795000</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>75645612</v>
+        <v>64745634</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>17</v>
@@ -2347,24 +2355,30 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>111669795</v>
       </c>
-      <c r="E52" s="7" t="n">
-        <v>3</v>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" s="9" t="n">
-        <v>68020787</v>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I52" s="7" t="n">
         <v>14</v>
@@ -3320,13 +3334,13 @@
         <v>156</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>1481524170</v>
+        <v>1487886270</v>
       </c>
       <c r="E76" s="7" t="n">
         <v>27</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>218178226</v>
+        <v>221823226</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>27</v>
@@ -3338,7 +3352,7 @@
         <v>129</v>
       </c>
       <c r="J76" s="9" t="n">
-        <v>1263345944</v>
+        <v>1266063044</v>
       </c>
     </row>
     <row r="77" ht="45" customHeight="1">
@@ -3349,28 +3363,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3945</v>
+        <v>3914</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32506512765</v>
+        <v>32592278796</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>458</v>
+        <v>427</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6695984642</v>
+        <v>6779033573</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>458</v>
+        <v>427</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>9494403177.6</v>
+        <v>6239819029.6</v>
       </c>
       <c r="I77" s="12" t="n">
         <v>3487</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>25810528123</v>
+        <v>25813245223</v>
       </c>
     </row>
   </sheetData>
@@ -3791,13 +3805,13 @@
         <v>5</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>413165330</v>
+        <v>428765330</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>261110330</v>
+        <v>276710330</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>3</v>
@@ -4592,28 +4606,28 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>1346095756</v>
+        <v>1566751699</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>1004886595</v>
+        <v>1225542538</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>852531955</v>
+        <v>896262562</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>852531955</v>
+        <v>896262562</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>4</v>
@@ -4834,28 +4848,28 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>388286000</v>
+        <v>538286000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>138750000</v>
+        <v>288750000</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>138306000</v>
+        <v>288306000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>138306000</v>
+        <v>288306000</v>
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
@@ -5570,28 +5584,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>523391100</v>
+        <v>595373450</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>345935300</v>
+        <v>417917650</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>187868022</v>
+        <v>198768000</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>187868022</v>
+        <v>198768000</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -6034,40 +6048,28 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>319983894</v>
-      </c>
-      <c r="E52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>660566066</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>340582172</v>
+      </c>
+      <c r="G52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>68020787</v>
+      </c>
+      <c r="I52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J52" s="9" t="n">
+        <v>68020787</v>
       </c>
       <c r="K52" s="10" t="inlineStr">
         <is>
@@ -7534,28 +7536,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>820</v>
+        <v>827</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>97165936093</v>
+        <v>97964756558</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>64597687680</v>
+        <v>65396508145</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>63405540890.41</v>
+        <v>63678192262.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>37278516146.02</v>
+        <v>37551167518.02</v>
       </c>
       <c r="K77" s="12" t="n">
         <v>12</v>
@@ -8369,28 +8371,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>26735477939</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>26735477939</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>26395646241</v>
+      </c>
+      <c r="I17" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="D17" s="11" t="n">
-        <v>25286544212</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="F17" s="11" t="n">
-        <v>25286544212</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>24599146241</v>
-      </c>
-      <c r="I17" s="4" t="n">
-        <v>21</v>
-      </c>
       <c r="J17" s="11" t="n">
-        <v>24599146241</v>
+        <v>26395646241</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8588,13 +8590,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8813,34 +8815,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>5652342335</v>
+        <v>48003814160</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>5281245056</v>
+        <v>47632716881</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>1854621974</v>
+        <v>2945468782</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -12011,34 +12013,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>136523671866</v>
+        <v>180959034603</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>99149023706</v>
+        <v>143584386443</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>67280217537.01</v>
+        <v>70262150313.01001</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>62831783737</v>
+        <v>65813716513</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>2915140258</v>
+        <v>4005987066</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>81</v>

</xml_diff>